<commit_message>
0.5.1 build, part: aura data path
</commit_message>
<xml_diff>
--- a/data/callings.xlsx
+++ b/data/callings.xlsx
@@ -653,7 +653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -663,6 +663,8 @@
     <col width="96" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -714,6 +716,11 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Enabled?</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Aura (15 ft, 15 ft allies, 15 ft enemies, add visible to pin it by default, or none)</t>
         </is>
       </c>
     </row>
@@ -929,7 +936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -939,6 +946,8 @@
     <col width="96" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -990,6 +999,11 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Enabled?</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Aura (15 ft, 15 ft allies, 15 ft enemies, add visible to pin it by default, or none)</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1238,6 +1252,8 @@
     <col width="96" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1289,6 +1305,11 @@
       <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Enabled?</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Aura (15 ft, 15 ft allies, 15 ft enemies, add visible to pin it by default, or none)</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1613,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1602,6 +1623,8 @@
     <col width="96" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1655,6 +1678,11 @@
           <t>Enabled?</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Aura (15 ft, 15 ft allies, 15 ft enemies, add visible to pin it by default, or none)</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="105" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -1685,6 +1713,11 @@
       </c>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>60 ft</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1868,7 +1901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1879,6 +1912,8 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1940,6 +1975,11 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Enabled?</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Aura (15 ft, 15 ft allies, 15 ft enemies, add visible to pin it by default, or none)</t>
         </is>
       </c>
     </row>

</xml_diff>